<commit_message>
Building and resource reports
</commit_message>
<xml_diff>
--- a/app/templates/report/edificios.xlsx
+++ b/app/templates/report/edificios.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\oimbra\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935E4375-54C8-4A2B-8AD4-00E29FC9F0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{702DD075-5DDB-4F31-9917-985D2315265A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Valoraciones" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Edificios!$A$2:$AG$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Edificios!$A$2:$AH$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Valoraciones!$A$2:$I$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
   <si>
     <t>Código</t>
   </si>
@@ -148,6 +148,9 @@
   </si>
   <si>
     <t>Histórico de valoraciones</t>
+  </si>
+  <si>
+    <t>Referencia catastral</t>
   </si>
 </sst>
 </file>
@@ -717,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AG3"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5546875" style="1" bestFit="1" customWidth="1"/>
@@ -727,28 +730,28 @@
     <col min="5" max="5" width="13.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="35.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.5546875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="33.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="18.6640625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="12" style="1" customWidth="1"/>
-    <col min="15" max="17" width="15.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="12" style="1" customWidth="1"/>
-    <col min="19" max="21" width="15.77734375" style="1" customWidth="1"/>
-    <col min="22" max="22" width="12" style="1" customWidth="1"/>
-    <col min="23" max="23" width="15.77734375" style="1" customWidth="1"/>
-    <col min="24" max="27" width="30.88671875" style="1" customWidth="1"/>
-    <col min="28" max="28" width="50.88671875" style="1" customWidth="1"/>
-    <col min="29" max="33" width="14.6640625" style="1" customWidth="1"/>
-    <col min="34" max="16384" width="24.88671875" style="1"/>
+    <col min="8" max="9" width="32.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="33.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="18.6640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="12" style="1" customWidth="1"/>
+    <col min="16" max="18" width="15.77734375" style="1" customWidth="1"/>
+    <col min="19" max="19" width="12" style="1" customWidth="1"/>
+    <col min="20" max="22" width="15.77734375" style="1" customWidth="1"/>
+    <col min="23" max="23" width="12" style="1" customWidth="1"/>
+    <col min="24" max="24" width="15.77734375" style="1" customWidth="1"/>
+    <col min="25" max="28" width="30.88671875" style="1" customWidth="1"/>
+    <col min="29" max="29" width="50.88671875" style="1" customWidth="1"/>
+    <col min="30" max="34" width="14.6640625" style="1" customWidth="1"/>
+    <col min="35" max="16384" width="24.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:33" s="8" customFormat="1" ht="25.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" s="8" customFormat="1" ht="25.2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -771,85 +774,88 @@
         <v>5</v>
       </c>
       <c r="H2" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="J2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="K2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="L2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="M2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="N2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="11" t="s">
+      <c r="O2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="P2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="Q2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="R2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="S2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="S2" s="9" t="s">
+      <c r="T2" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="9" t="s">
+      <c r="U2" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="V2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V2" s="11" t="s">
+      <c r="W2" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="W2" s="9" t="s">
+      <c r="X2" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="X2" s="11" t="s">
+      <c r="Y2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="Y2" s="9" t="s">
+      <c r="Z2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="Z2" s="9" t="s">
+      <c r="AA2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="AA2" s="9" t="s">
+      <c r="AB2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="AB2" s="9" t="s">
+      <c r="AC2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="AC2" s="9" t="s">
+      <c r="AD2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="AD2" s="9" t="s">
+      <c r="AE2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="AE2" s="9" t="s">
+      <c r="AF2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="AF2" s="9" t="s">
+      <c r="AG2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="AG2" s="9" t="s">
+      <c r="AH2" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:33" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -860,43 +866,44 @@
       <c r="F3" s="3"/>
       <c r="G3" s="4"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="13" t="s">
+      <c r="M3" s="3"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O3" s="10"/>
       <c r="P3" s="10"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="13" t="s">
+      <c r="Q3" s="10"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="S3" s="10"/>
       <c r="T3" s="10"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="13" t="s">
+      <c r="U3" s="10"/>
+      <c r="V3" s="12"/>
+      <c r="W3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="W3" s="12"/>
-      <c r="X3" s="15"/>
-      <c r="Y3" s="5"/>
+      <c r="X3" s="12"/>
+      <c r="Y3" s="15"/>
       <c r="Z3" s="5"/>
       <c r="AA3" s="5"/>
       <c r="AB3" s="5"/>
-      <c r="AC3" s="3"/>
+      <c r="AC3" s="5"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AG2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="R3:U99999">
+  <autoFilter ref="A2:AH2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="S3:V99999">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>EDATE($R3,6)&lt;TODAY()</formula>
+      <formula>EDATE($S3,6)&lt;TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>